<commit_message>
V0.1 with variables contained within the model workspace
PID tables still need adjusting for TV!
</commit_message>
<xml_diff>
--- a/Control Algorithms/Stacey's Old Work (FB25)/v0_signal_names.xlsx
+++ b/Control Algorithms/Stacey's Old Work (FB25)/v0_signal_names.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GITHUB\FB26_Controls\Control Algorithms\Stacey's Old Work (FB25)\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{708C0F74-36BE-4CD1-8630-D763724CA772}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0F03686-49C4-419B-B88D-115EBF95496D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6408ACC7-8B01-4673-96AC-DFD7837C0511}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{6408ACC7-8B01-4673-96AC-DFD7837C0511}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Signal Names" sheetId="1" r:id="rId1"/>
+    <sheet name="Variable Names" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="109">
   <si>
     <t>Signal</t>
   </si>
@@ -198,6 +199,171 @@
   </si>
   <si>
     <t>CMD_TV_delta</t>
+  </si>
+  <si>
+    <t>Variable Name</t>
+  </si>
+  <si>
+    <t>Variable</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>Unit</t>
+  </si>
+  <si>
+    <t>Maximum Motor Torque Output</t>
+  </si>
+  <si>
+    <t>Tmax</t>
+  </si>
+  <si>
+    <t>Note</t>
+  </si>
+  <si>
+    <t>The maximum possible torque output isnt availible at all times.</t>
+  </si>
+  <si>
+    <t>Gearbox Ratio</t>
+  </si>
+  <si>
+    <t>GR</t>
+  </si>
+  <si>
+    <t>FB26 gearbox ratio is 14.14 motor revs per 1 wheel rev</t>
+  </si>
+  <si>
+    <t>Required Yaw Moment to Rear Axle Torque Difference</t>
+  </si>
+  <si>
+    <t>Mz_to_CMD_TV_delta</t>
+  </si>
+  <si>
+    <t>mu</t>
+  </si>
+  <si>
+    <t>The coefficient of friction between the tires and the road</t>
+  </si>
+  <si>
+    <t>Nm/Nm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">g </t>
+  </si>
+  <si>
+    <t>m/s^2</t>
+  </si>
+  <si>
+    <t>Coefficient of Friction</t>
+  </si>
+  <si>
+    <t>Gravitational Constant</t>
+  </si>
+  <si>
+    <t>CG Height</t>
+  </si>
+  <si>
+    <t>h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">m </t>
+  </si>
+  <si>
+    <t>Track width</t>
+  </si>
+  <si>
+    <t>t</t>
+  </si>
+  <si>
+    <t>m</t>
+  </si>
+  <si>
+    <t>Wheelbase</t>
+  </si>
+  <si>
+    <t>L</t>
+  </si>
+  <si>
+    <t>Izz</t>
+  </si>
+  <si>
+    <t>kgm^2</t>
+  </si>
+  <si>
+    <t>Feed Forward Gain</t>
+  </si>
+  <si>
+    <t>Yaw Inertia</t>
+  </si>
+  <si>
+    <t>Ffgain</t>
+  </si>
+  <si>
+    <t>The gain added to the desired yaw moment signal in torque vectoring</t>
+  </si>
+  <si>
+    <t>A dynamic look up table for PID gain values based on velocity</t>
+  </si>
+  <si>
+    <t>Kp</t>
+  </si>
+  <si>
+    <t>Ki</t>
+  </si>
+  <si>
+    <t>Kd</t>
+  </si>
+  <si>
+    <t>Kn</t>
+  </si>
+  <si>
+    <t>Unsure on what these are or should be</t>
+  </si>
+  <si>
+    <t>The amount of rear axle torque difference (left to right) required to achieve a given yaw moment. Unsure on the value it needs to be.</t>
+  </si>
+  <si>
+    <t>Feedback Gain</t>
+  </si>
+  <si>
+    <t>The gain added to the TV PID controllers signal</t>
+  </si>
+  <si>
+    <t>FBgain</t>
+  </si>
+  <si>
+    <t>TV PID P table</t>
+  </si>
+  <si>
+    <t>TV PID I table</t>
+  </si>
+  <si>
+    <t>TV PID D table</t>
+  </si>
+  <si>
+    <t>TV PID N table</t>
+  </si>
+  <si>
+    <t>TV PID D Gain</t>
+  </si>
+  <si>
+    <t>TV PID N Gain</t>
+  </si>
+  <si>
+    <t>TV PID P Gain</t>
+  </si>
+  <si>
+    <t>TV PID I Gain</t>
+  </si>
+  <si>
+    <t>Desired Slip Ratio</t>
+  </si>
+  <si>
+    <t>kappa_desired</t>
+  </si>
+  <si>
+    <t>The desired rear wheel slip ratio</t>
   </si>
 </sst>
 </file>
@@ -863,4 +1029,363 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29BE85F6-1FC1-42B5-84CF-C5ABF5A75E2B}">
+  <dimension ref="A1:E21"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="48.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="117.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C2">
+        <v>21</v>
+      </c>
+      <c r="D2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E2" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C3">
+        <v>14.14</v>
+      </c>
+      <c r="D3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E3" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>65</v>
+      </c>
+      <c r="B4" t="s">
+        <v>66</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4" t="s">
+        <v>69</v>
+      </c>
+      <c r="E4" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>72</v>
+      </c>
+      <c r="B5" t="s">
+        <v>67</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E5" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>73</v>
+      </c>
+      <c r="B6" t="s">
+        <v>70</v>
+      </c>
+      <c r="C6">
+        <v>9.81</v>
+      </c>
+      <c r="D6" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>74</v>
+      </c>
+      <c r="B7" t="s">
+        <v>75</v>
+      </c>
+      <c r="C7">
+        <v>0.22500000000000001</v>
+      </c>
+      <c r="D7" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>77</v>
+      </c>
+      <c r="B8" t="s">
+        <v>78</v>
+      </c>
+      <c r="C8">
+        <v>1.2</v>
+      </c>
+      <c r="D8" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>80</v>
+      </c>
+      <c r="B9" t="s">
+        <v>81</v>
+      </c>
+      <c r="C9">
+        <v>1.53</v>
+      </c>
+      <c r="D9" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>85</v>
+      </c>
+      <c r="B10" t="s">
+        <v>82</v>
+      </c>
+      <c r="C10">
+        <v>80</v>
+      </c>
+      <c r="D10" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>84</v>
+      </c>
+      <c r="B11" t="s">
+        <v>86</v>
+      </c>
+      <c r="C11">
+        <v>1</v>
+      </c>
+      <c r="D11" t="s">
+        <v>4</v>
+      </c>
+      <c r="E11" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>98</v>
+      </c>
+      <c r="B12" t="s">
+        <v>4</v>
+      </c>
+      <c r="C12" t="s">
+        <v>4</v>
+      </c>
+      <c r="D12" t="s">
+        <v>4</v>
+      </c>
+      <c r="E12" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>99</v>
+      </c>
+      <c r="B13" t="s">
+        <v>4</v>
+      </c>
+      <c r="C13" t="s">
+        <v>4</v>
+      </c>
+      <c r="D13" t="s">
+        <v>4</v>
+      </c>
+      <c r="E13" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>100</v>
+      </c>
+      <c r="B14" t="s">
+        <v>4</v>
+      </c>
+      <c r="C14" t="s">
+        <v>4</v>
+      </c>
+      <c r="D14" t="s">
+        <v>4</v>
+      </c>
+      <c r="E14" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>101</v>
+      </c>
+      <c r="B15" t="s">
+        <v>4</v>
+      </c>
+      <c r="C15" t="s">
+        <v>4</v>
+      </c>
+      <c r="D15" t="s">
+        <v>4</v>
+      </c>
+      <c r="E15" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>104</v>
+      </c>
+      <c r="B16" t="s">
+        <v>89</v>
+      </c>
+      <c r="C16">
+        <v>1</v>
+      </c>
+      <c r="D16" t="s">
+        <v>4</v>
+      </c>
+      <c r="E16" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>105</v>
+      </c>
+      <c r="B17" t="s">
+        <v>90</v>
+      </c>
+      <c r="C17">
+        <v>1</v>
+      </c>
+      <c r="D17" t="s">
+        <v>4</v>
+      </c>
+      <c r="E17" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>102</v>
+      </c>
+      <c r="B18" t="s">
+        <v>91</v>
+      </c>
+      <c r="C18">
+        <v>1</v>
+      </c>
+      <c r="D18" t="s">
+        <v>4</v>
+      </c>
+      <c r="E18" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>103</v>
+      </c>
+      <c r="B19" t="s">
+        <v>92</v>
+      </c>
+      <c r="C19">
+        <v>1</v>
+      </c>
+      <c r="D19" t="s">
+        <v>4</v>
+      </c>
+      <c r="E19" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>95</v>
+      </c>
+      <c r="B20" t="s">
+        <v>97</v>
+      </c>
+      <c r="C20">
+        <v>1</v>
+      </c>
+      <c r="D20" t="s">
+        <v>4</v>
+      </c>
+      <c r="E20" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>106</v>
+      </c>
+      <c r="B21" t="s">
+        <v>107</v>
+      </c>
+      <c r="C21">
+        <v>0.2</v>
+      </c>
+      <c r="D21" t="s">
+        <v>4</v>
+      </c>
+      <c r="E21" t="s">
+        <v>108</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
V0.1 with updated TV PID controller gain tables
</commit_message>
<xml_diff>
--- a/Control Algorithms/Stacey's Old Work (FB25)/v0_signal_names.xlsx
+++ b/Control Algorithms/Stacey's Old Work (FB25)/v0_signal_names.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GITHUB\FB26_Controls\Control Algorithms\Stacey's Old Work (FB25)\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0F03686-49C4-419B-B88D-115EBF95496D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF7943AC-CEDC-4A1E-BF7D-2348BA4D478E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{6408ACC7-8B01-4673-96AC-DFD7837C0511}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="120">
   <si>
     <t>Signal</t>
   </si>
@@ -364,6 +364,39 @@
   </si>
   <si>
     <t>The desired rear wheel slip ratio</t>
+  </si>
+  <si>
+    <t>Pgain</t>
+  </si>
+  <si>
+    <t>Igain</t>
+  </si>
+  <si>
+    <t>Dgain</t>
+  </si>
+  <si>
+    <t>Ngain</t>
+  </si>
+  <si>
+    <t>TV PID Velocity Vector</t>
+  </si>
+  <si>
+    <t>vx_vector</t>
+  </si>
+  <si>
+    <t>The velocity vector for the TV PID gain tables</t>
+  </si>
+  <si>
+    <t>TV PID Back Calculation Coefficient</t>
+  </si>
+  <si>
+    <t>Kb</t>
+  </si>
+  <si>
+    <t>The coefficient for the antiwindup method (back calculation)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">m/s </t>
   </si>
 </sst>
 </file>
@@ -1033,7 +1066,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29BE85F6-1FC1-42B5-84CF-C5ABF5A75E2B}">
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="48.140625" bestFit="1" customWidth="1"/>
@@ -1220,7 +1253,7 @@
         <v>98</v>
       </c>
       <c r="B12" t="s">
-        <v>4</v>
+        <v>109</v>
       </c>
       <c r="C12" t="s">
         <v>4</v>
@@ -1237,7 +1270,7 @@
         <v>99</v>
       </c>
       <c r="B13" t="s">
-        <v>4</v>
+        <v>110</v>
       </c>
       <c r="C13" t="s">
         <v>4</v>
@@ -1254,7 +1287,7 @@
         <v>100</v>
       </c>
       <c r="B14" t="s">
-        <v>4</v>
+        <v>111</v>
       </c>
       <c r="C14" t="s">
         <v>4</v>
@@ -1271,7 +1304,7 @@
         <v>101</v>
       </c>
       <c r="B15" t="s">
-        <v>4</v>
+        <v>112</v>
       </c>
       <c r="C15" t="s">
         <v>4</v>
@@ -1291,7 +1324,7 @@
         <v>89</v>
       </c>
       <c r="C16">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="D16" t="s">
         <v>4</v>
@@ -1308,7 +1341,7 @@
         <v>90</v>
       </c>
       <c r="C17">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D17" t="s">
         <v>4</v>
@@ -1325,7 +1358,7 @@
         <v>91</v>
       </c>
       <c r="C18">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D18" t="s">
         <v>4</v>
@@ -1383,6 +1416,40 @@
       </c>
       <c r="E21" t="s">
         <v>108</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>113</v>
+      </c>
+      <c r="B22" t="s">
+        <v>114</v>
+      </c>
+      <c r="C22" t="s">
+        <v>4</v>
+      </c>
+      <c r="D22" t="s">
+        <v>119</v>
+      </c>
+      <c r="E22" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>116</v>
+      </c>
+      <c r="B23" t="s">
+        <v>117</v>
+      </c>
+      <c r="C23">
+        <v>5</v>
+      </c>
+      <c r="D23" t="s">
+        <v>4</v>
+      </c>
+      <c r="E23" t="s">
+        <v>118</v>
       </c>
     </row>
   </sheetData>

</xml_diff>